<commit_message>
update document generation. now locale dependent.
</commit_message>
<xml_diff>
--- a/src/Services/Main/Main.Application/Document/Sales/SingleSale.xlsx
+++ b/src/Services/Main/Main.Application/Document/Sales/SingleSale.xlsx
@@ -8,8 +8,11 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Продажа" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sale" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="Items">'Sale'!$A$15:$H$16</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -22,7 +25,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
-    <t xml:space="preserve">ДОКУМЕНТ ПРОДАЖИ</t>
+    <t xml:space="preserve">SALES DOCUMENT</t>
   </si>
   <si>
     <t xml:space="preserve">{{OrganizationName}}</t>
@@ -31,10 +34,10 @@
     <t xml:space="preserve">{{StorageCode}} · {{CurrencyCode}}</t>
   </si>
   <si>
-    <t xml:space="preserve">ПРОДАЖА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДАТА ПРОДАЖИ</t>
+    <t xml:space="preserve">SALE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SALE DATE</t>
   </si>
   <si>
     <t xml:space="preserve">№ {{Id}}</t>
@@ -43,97 +46,97 @@
     <t xml:space="preserve">{{SaleDatetime}}</t>
   </si>
   <si>
-    <t xml:space="preserve">Транзакция: {{TransactionId}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Статус: {{State}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПОКУПАТЕЛЬ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДЕТАЛИ</t>
+    <t xml:space="preserve">Transaction: {{TransactionId}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status: {{State}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUYER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DETAILS</t>
   </si>
   <si>
     <t xml:space="preserve">{{BuyerName}}</t>
   </si>
   <si>
-    <t xml:space="preserve">Склад</t>
+    <t xml:space="preserve">Warehouse</t>
   </si>
   <si>
     <t xml:space="preserve">{{StorageCode}}</t>
   </si>
   <si>
-    <t xml:space="preserve">Валюта</t>
+    <t xml:space="preserve">Currency</t>
   </si>
   <si>
     <t xml:space="preserve">{{CurrencyCode}}  {{CurrencySign}}</t>
   </si>
   <si>
-    <t xml:space="preserve">ПОЗИЦИИ</t>
+    <t xml:space="preserve">ITEMS</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Артикул</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наименование</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кол-во</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Скидка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сумма</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Комментарий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.ProductId}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.Sku}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.ProductName}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.Count}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.Price}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.Discount}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.TotalSum}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{Items.Comment}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ИТОГО</t>
+    <t xml:space="preserve">SKU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.ProductId}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.Sku}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.ProductName}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.Count}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.Price}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.Discount}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.TotalSum}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{item.Comment}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
     <t xml:space="preserve">{{TotalSum}} {{CurrencySign}}</t>
   </si>
   <si>
-    <t xml:space="preserve">КОММЕНТАРИЙ</t>
+    <t xml:space="preserve">COMMENT</t>
   </si>
   <si>
     <t xml:space="preserve">{{Comment}}</t>
   </si>
   <si>
-    <t xml:space="preserve">Документ сформирован автоматически</t>
+    <t xml:space="preserve">Generated automatically</t>
   </si>
   <si>
     <t xml:space="preserve">Transaction ID: {{TransactionId}}</t>
@@ -143,8 +146,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -382,7 +386,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -489,6 +493,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -819,7 +827,7 @@
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G6" s="9"/>

</xml_diff>